<commit_message>
Hierarchical category filter, category-page timeout fix, typo fix, card polish
</commit_message>
<xml_diff>
--- a/data/channels_complete.xlsx
+++ b/data/channels_complete.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Channels Youtube" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels Youtube" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11568,7 +11568,7 @@
       </c>
       <c r="F279" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H279" s="8" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="F280" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H280" s="8" t="inlineStr">
@@ -11634,7 +11634,7 @@
       </c>
       <c r="F281" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H281" s="8" t="inlineStr">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="F282" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H282" s="8" t="inlineStr">
@@ -11700,7 +11700,7 @@
       </c>
       <c r="F283" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H283" s="8" t="inlineStr">
@@ -11733,7 +11733,7 @@
       </c>
       <c r="F284" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H284" s="8" t="inlineStr">
@@ -11766,7 +11766,7 @@
       </c>
       <c r="F285" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H285" s="8" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="F286" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H286" s="8" t="inlineStr">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="F287" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H287" s="8" t="inlineStr">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="F288" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H288" s="8" t="inlineStr">
@@ -11898,7 +11898,7 @@
       </c>
       <c r="F289" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H289" s="8" t="inlineStr">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="F290" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H290" s="8" t="inlineStr">
@@ -11964,7 +11964,7 @@
       </c>
       <c r="F291" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H291" s="8" t="inlineStr">
@@ -11997,7 +11997,7 @@
       </c>
       <c r="F292" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H292" s="8" t="inlineStr">
@@ -12030,7 +12030,7 @@
       </c>
       <c r="F293" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H293" s="8" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="F294" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H294" s="8" t="inlineStr">
@@ -12096,7 +12096,7 @@
       </c>
       <c r="F295" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H295" s="8" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="F296" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H296" s="8" t="inlineStr">
@@ -12162,7 +12162,7 @@
       </c>
       <c r="F297" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H297" s="8" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="F298" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H298" s="8" t="inlineStr">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="F299" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H299" s="8" t="inlineStr">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="F300" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H300" s="8" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="F301" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H301" s="8" t="inlineStr">
@@ -12327,7 +12327,7 @@
       </c>
       <c r="F302" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H302" s="8" t="inlineStr">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="F303" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H303" s="8" t="inlineStr">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="F304" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H304" s="8" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
       <c r="F305" s="21" t="inlineStr">
         <is>
-          <t>Incluencer Cycling</t>
+          <t>Influencer Cycling</t>
         </is>
       </c>
       <c r="H305" s="8" t="inlineStr">

</xml_diff>